<commit_message>
PAUSED (task178): the moved window's owner and forcing event redrawn (a paper mill, the 2027 in-water season), card re-registered, stage 3 green, waiting on the readers and judge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task178/golden/sauer_crossing_design_flow.xlsx
+++ b/task178/golden/sauer_crossing_design_flow.xlsx
@@ -29,7 +29,7 @@
     <t>Sauer pipe bridge replacement: design discharge and waterway alternative</t>
   </si>
   <si>
-    <t>TUM-02 Tumwick River near Sauer, annual peaks of water years 1980 to 2025, Design Standard 4.2</t>
+    <t>TUM-02 Tumwick River near Sauer, annual peaks of water years 1980 to 2025, Engineering Standard 4.2</t>
   </si>
   <si>
     <t>Alternative to carry forward</t>
@@ -152,7 +152,7 @@
     <t>Annual peaks are the largest instantaneous stage of each water year (1 October to 30 September): the register for 1980 to 2015, the 15-minute record for 2016 to 2025.</t>
   </si>
   <si>
-    <t>Frequency analysis per Design Standard 4.2 (issue 3). The design discharge is reported to the nearest 1,000 cfs.</t>
+    <t>Frequency analysis per Engineering Standard 4.2 (issue 3). The design discharge is reported to the nearest 1,000 cfs.</t>
   </si>
   <si>
     <t>Work windows: readings taken while a hydrographer was on site are left out (visit log times are local); the controller offset of 0.47 ft is removed from 11 June to 27 August 2025.</t>

</xml_diff>